<commit_message>
Ronde 5: min. artikelen per binnendoos en bestaande buitendoos zonder binnendoos
- "Min. artikelen per binnendoos" overal, standaard 2 (formulier, nieuw
  artikel, lege importcel); artikel zonder binnendoos blijft 1. Afgeleide
  aantallen artikelen staan met "min." in resultaten en PDF.
- Bestaande buitendoos: vinkje "Binnendoos opgeven" (standaard uit).
  Zonder binnendoos vul je alleen maten, gevuld gewicht (verplicht) en
  eventueel artikelen per buitendoos in; resultaten en PDF tellen
  artikelen, het PDF toont "Geen binnendoos".
- Import herkent oude en nieuwe kop; voorbeeldbestand bijgewerkt.
- Ontwerp V1.6, besluiten ronde 5 (#61, #62), README en tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kLLQRGDJYD9iRUtGgdMVZ
</commit_message>
<xml_diff>
--- a/public/voorbeeld-artikelen.xlsx
+++ b/public/voorbeeld-artikelen.xlsx
@@ -455,7 +455,7 @@
     <col width="25" customWidth="1" style="2" min="3" max="3"/>
     <col width="24" customWidth="1" style="2" min="4" max="4"/>
     <col width="36" customWidth="1" style="3" min="5" max="5"/>
-    <col width="31" customWidth="1" style="2" min="6" max="6"/>
+    <col width="36" customWidth="1" style="2" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -487,7 +487,7 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Aantal artikelen per binnendoos</t>
+          <t>Min. aantal artikelen per binnendoos</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
@@ -501,7 +501,7 @@
     <dataValidation sqref="B2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen geldige waarde" error="Vul een getal groter dan 0 in." type="decimal" errorStyle="warning" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen geldig aantal" error="Vul een geheel getal van minstens 1 in, of laat de cel leeg (= 1)." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
+    <dataValidation sqref="F2:F10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen geldig aantal" error="Vul een geheel getal van minstens 1 in, of laat de cel leeg (= 2)." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
@@ -640,12 +640,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Aantal artikelen per binnendoos</t>
+          <t>Min. aantal artikelen per binnendoos</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Hoeveel artikelen er in één binnendoos zitten, als geheel getal. Mag leeg blijven: leeg = 1.</t>
+          <t>Hoeveel artikelen er minstens in één binnendoos zitten, als geheel getal. Mag leeg blijven: leeg = 2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ronde 8: zachte vormregel, vast aantal artikelen per binnendoos en kantelbaar in de import
- #66: nieuwe standaardvormregel zacht. Een ontworpen buitendoos mag hoger zijn
  dan breed, tot 2 × de breedte (instelbaar), en wint alleen bij minstens 10%
  meer binnendozen per drager dan de platte voorkeursoptie (de uitkomst van
  breedte). Wint zo'n doos, dan staat die platte uitkomst als kaart "Niet hoger
  dan breed" in de top drie. Instellingen versie 3: breedte gaat eenmalig naar
  zacht.
- #67: "Artikelen per binnendoos" is weer een vast aantal; geen "min." meer in
  resultaten en PDF.
- #68: de Excel-import van artikelen leest Kantelbaar, L mag verticaal en
  B mag verticaal; het voorbeeldbestand heeft die kolommen en een werkblad
  Voorbeeld.
- Tests, besluiten ronde 8, functioneel ontwerp V1.9 en README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kLLQRGDJYD9iRUtGgdMVZ
</commit_message>
<xml_diff>
--- a/public/voorbeeld-artikelen.xlsx
+++ b/public/voorbeeld-artikelen.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artikelen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Uitleg" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voorbeeld" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -455,8 +456,11 @@
     <col width="25" customWidth="1" style="2" min="3" max="3"/>
     <col width="24" customWidth="1" style="2" min="4" max="4"/>
     <col width="36" customWidth="1" style="3" min="5" max="5"/>
-    <col width="36" customWidth="1" style="2" min="6" max="6"/>
+    <col width="26" customWidth="1" style="2" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,7 +491,7 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Min. aantal artikelen per binnendoos</t>
+          <t>Artikelen per binnendoos</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
@@ -495,14 +499,32 @@
           <t>Omschrijving</t>
         </is>
       </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Kantelbaar (ja/nee)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>L mag verticaal (ja/nee)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>B mag verticaal (ja/nee)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="B2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen geldige waarde" error="Vul een getal groter dan 0 in." type="decimal" errorStyle="warning" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen geldig aantal" error="Vul een geheel getal van minstens 1 in, of laat de cel leeg (= 2)." type="whole" errorStyle="warning" operator="greaterThanOrEqual">
       <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:J10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Geen ja of nee" error="Vul ja of nee in, of laat de cel leeg (= nee)." type="list" errorStyle="warning">
+      <formula1>"ja,nee"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -515,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -640,12 +662,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Min. aantal artikelen per binnendoos</t>
+          <t>Artikelen per binnendoos</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Hoeveel artikelen er minstens in één binnendoos zitten, als geheel getal. Mag leeg blijven: leeg = 2.</t>
+          <t>Hoeveel artikelen er in één binnendoos zitten, als geheel getal. Mag leeg blijven: leeg = 2.</t>
         </is>
       </c>
     </row>
@@ -666,52 +688,318 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Kantelbaar (ja/nee)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Ja als de binnendoos op zijn kant mag staan, anders nee. Mag leeg blijven: leeg = nee. Bij ja moet L of B (of allebei) verticaal mogen.</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>L mag verticaal (ja/nee)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Ja als de binnendoos zo mag staan dat de lengte verticaal is. Alleen bij kantelbaar ja. Leeg = nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>B mag verticaal (ja/nee)</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Ja als de binnendoos zo mag staan dat de breedte verticaal is. Alleen bij kantelbaar ja. Leeg = nee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Goed om te weten</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>- Laat de eerste rij met de kolomnamen staan: de app herkent daaraan de kolommen en de eenheden. Vul vanaf rij 2 één artikel per rij in.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>- Lengtes in millimeters (mm), gewicht in kilogram (kg) inclusief inhoud.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>- De app kiest bij het importeren standaard het eerste werkblad (Artikelen).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- Een nieuw artikelnummer wordt als nieuw artikel aangemaakt. Een bestaand artikel wordt alleen overschreven als je de wijziging in de app bevestigt.</t>
+          <t>- Laat de eerste rij met de kolomnamen staan: de app herkent daaraan de kolommen en de eenheden. Vul vanaf rij 2 één artikel per rij in.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>- Kantelbaar en welke as verticaal mag staan stel je daarna per artikel in op het tabblad Artikelen.</t>
+          <t>- Lengtes in millimeters (mm), gewicht in kilogram (kg) inclusief inhoud.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>- De app kiest bij het importeren standaard het eerste werkblad (Artikelen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- Een nieuw artikelnummer wordt als nieuw artikel aangemaakt. Een bestaand artikel wordt alleen overschreven als je de wijziging in de app bevestigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>- Voor ja en nee mag ook: j en n, yes en no, x (= ja), 1 en 0, of waar en onwaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>- Laat je de kolom Kantelbaar weg, dan zijn nieuwe artikelen niet kantelbaar en blijven de kantelrechten van bestaande artikelen zoals ze zijn. Je kunt ze ook later per artikel aanpassen op het tabblad Artikelen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>- Het werkblad Voorbeeld toont drie ingevulde rijen. Vul je eigen artikelen in op het werkblad Artikelen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>- Importeren gaat via het tabblad Excel-import.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="1" min="1" max="1"/>
+    <col width="24" customWidth="1" style="2" min="2" max="2"/>
+    <col width="25" customWidth="1" style="2" min="3" max="3"/>
+    <col width="24" customWidth="1" style="2" min="4" max="4"/>
+    <col width="36" customWidth="1" style="3" min="5" max="5"/>
+    <col width="26" customWidth="1" style="2" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Artikelcode</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Lengte binnendoos (mm)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Breedte binnendoos (mm)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Hoogte binnendoos (mm)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Gewicht binnendoos incl. inhoud (kg)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Artikelen per binnendoos</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Omschrijving</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Kantelbaar (ja/nee)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>L mag verticaal (ja/nee)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>B mag verticaal (ja/nee)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VOORBEELD-1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>300</v>
+      </c>
+      <c r="C2" t="n">
+        <v>200</v>
+      </c>
+      <c r="D2" t="n">
+        <v>150</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kop en schotel</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nee</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nee</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VOORBEELD-2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>400</v>
+      </c>
+      <c r="C3" t="n">
+        <v>250</v>
+      </c>
+      <c r="D3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Vaas</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VOORBEELD-3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>350</v>
+      </c>
+      <c r="C4" t="n">
+        <v>300</v>
+      </c>
+      <c r="D4" t="n">
+        <v>200</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Bordenset</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ja</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ronde 9 (tussenstand): import, kantelen bij vierkante doos, verband in de buurt van een blok
- Import: bij Kantelbaar ja is een lege askolom ja; een lege Kantelbaar met
  ja bij L of B maakt de doos kantelbaar voor die as. Foute rijen krijgen een
  waarschuwing boven de tabel.
- standen(): een gekantelde stand met dezelfde maten als een eerdere stand
  valt weg (bijvoorbeeld B = H).
- Verband telt alleen als elke doos voor minstens de min. ondersteuning op de
  laag eronder rust en elke laag hoogstens de max. inham (standaard 5%) aan
  de rand van het blok leeg laat. Nieuwe instelling "Max. inham per laag bij
  verband".
- Nieuwe tests in tests/ronde9.test.ts. De bestaande tests die nog op het
  oude verband rekenen, volgen in een volgende commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kLLQRGDJYD9iRUtGgdMVZ
</commit_message>
<xml_diff>
--- a/public/voorbeeld-artikelen.xlsx
+++ b/public/voorbeeld-artikelen.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Ja als de binnendoos op zijn kant mag staan, anders nee. Mag leeg blijven: leeg = nee. Bij ja moet L of B (of allebei) verticaal mogen.</t>
+          <t>Ja als de binnendoos op zijn kant mag staan, anders nee. Mag leeg blijven: leeg = nee, tenzij bij L of B ja staat. Bij ja mogen L en B allebei verticaal, behalve als er bij L of B nee staat.</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Ja als de binnendoos zo mag staan dat de lengte verticaal is. Alleen bij kantelbaar ja. Leeg = nee.</t>
+          <t>Ja als de binnendoos zo mag staan dat de lengte verticaal is, nee als dat niet mag. Leeg = ja bij kantelbaar ja, anders nee.</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Ja als de binnendoos zo mag staan dat de breedte verticaal is. Alleen bij kantelbaar ja. Leeg = nee.</t>
+          <t>Ja als de binnendoos zo mag staan dat de breedte verticaal is, nee als dat niet mag. Leeg = ja bij kantelbaar ja, anders nee.</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- Een nieuw artikelnummer wordt als nieuw artikel aangemaakt. Een bestaand artikel wordt alleen overschreven als je de wijziging in de app bevestigt.</t>
+          <t>- Een nieuw artikelnummer wordt als nieuw artikel aangemaakt. Een bestaand artikel wordt alleen overschreven als je de wijziging in de app bevestigt. Een rij met een fout wordt niet geïmporteerd; de app toont de fout per rij.</t>
         </is>
       </c>
     </row>

</xml_diff>